<commit_message>
fix(financial-model): audit and resolve all formula references and cell formatting across all tabs
</commit_message>
<xml_diff>
--- a/PRISM_CFO_Financial_Model_v1.xlsx
+++ b/PRISM_CFO_Financial_Model_v1.xlsx
@@ -23,8 +23,8 @@
   <numFmts count="5">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
-    <numFmt numFmtId="166" formatCode="#,##0.0"/>
-    <numFmt numFmtId="167" formatCode="$#,##0.0"/>
+    <numFmt numFmtId="166" formatCode="$#,##0.0"/>
+    <numFmt numFmtId="167" formatCode="#,##0.0"/>
     <numFmt numFmtId="168" formatCode="0.0&quot;x&quot;"/>
   </numFmts>
   <fonts count="11">
@@ -213,6 +213,9 @@
     <xf numFmtId="3" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
@@ -245,13 +248,10 @@
     <xf numFmtId="164" fontId="9" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="9" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="3" fontId="8" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -267,10 +267,10 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="8" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="168" fontId="8" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -805,7 +805,7 @@
     <row r="13">
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>Monthly Routed Notional ($M)</t>
+          <t>Avg Monthly Volume / Desk ($M)</t>
         </is>
       </c>
       <c r="C13" s="12">
@@ -835,23 +835,23 @@
           <t>Annual Routed Notional ($M)</t>
         </is>
       </c>
-      <c r="C14" s="12">
+      <c r="C14" s="13">
         <f>'5-Year Pro-Forma'!C14</f>
         <v/>
       </c>
-      <c r="D14" s="12">
+      <c r="D14" s="13">
         <f>'5-Year Pro-Forma'!D14</f>
         <v/>
       </c>
-      <c r="E14" s="12">
+      <c r="E14" s="13">
         <f>'5-Year Pro-Forma'!E14</f>
         <v/>
       </c>
-      <c r="F14" s="12">
+      <c r="F14" s="13">
         <f>'5-Year Pro-Forma'!F14</f>
         <v/>
       </c>
-      <c r="G14" s="12">
+      <c r="G14" s="13">
         <f>'5-Year Pro-Forma'!G14</f>
         <v/>
       </c>
@@ -863,23 +863,23 @@
           <t>SaaS Subscription Revenue</t>
         </is>
       </c>
-      <c r="C16" s="12">
+      <c r="C16" s="13">
         <f>'5-Year Pro-Forma'!C21</f>
         <v/>
       </c>
-      <c r="D16" s="12">
+      <c r="D16" s="13">
         <f>'5-Year Pro-Forma'!D21</f>
         <v/>
       </c>
-      <c r="E16" s="12">
+      <c r="E16" s="13">
         <f>'5-Year Pro-Forma'!E21</f>
         <v/>
       </c>
-      <c r="F16" s="12">
+      <c r="F16" s="13">
         <f>'5-Year Pro-Forma'!F21</f>
         <v/>
       </c>
-      <c r="G16" s="12">
+      <c r="G16" s="13">
         <f>'5-Year Pro-Forma'!G21</f>
         <v/>
       </c>
@@ -890,23 +890,23 @@
           <t>Volume Routing Take-Rate</t>
         </is>
       </c>
-      <c r="C17" s="12">
+      <c r="C17" s="13">
         <f>'5-Year Pro-Forma'!C22</f>
         <v/>
       </c>
-      <c r="D17" s="12">
+      <c r="D17" s="13">
         <f>'5-Year Pro-Forma'!D22</f>
         <v/>
       </c>
-      <c r="E17" s="12">
+      <c r="E17" s="13">
         <f>'5-Year Pro-Forma'!E22</f>
         <v/>
       </c>
-      <c r="F17" s="12">
+      <c r="F17" s="13">
         <f>'5-Year Pro-Forma'!F22</f>
         <v/>
       </c>
-      <c r="G17" s="12">
+      <c r="G17" s="13">
         <f>'5-Year Pro-Forma'!G22</f>
         <v/>
       </c>
@@ -917,23 +917,23 @@
           <t>Premium Data &amp; SLA Feeds</t>
         </is>
       </c>
-      <c r="C18" s="12">
+      <c r="C18" s="13">
         <f>'5-Year Pro-Forma'!C23</f>
         <v/>
       </c>
-      <c r="D18" s="12">
+      <c r="D18" s="13">
         <f>'5-Year Pro-Forma'!D23</f>
         <v/>
       </c>
-      <c r="E18" s="12">
+      <c r="E18" s="13">
         <f>'5-Year Pro-Forma'!E23</f>
         <v/>
       </c>
-      <c r="F18" s="12">
+      <c r="F18" s="13">
         <f>'5-Year Pro-Forma'!F23</f>
         <v/>
       </c>
-      <c r="G18" s="12">
+      <c r="G18" s="13">
         <f>'5-Year Pro-Forma'!G23</f>
         <v/>
       </c>
@@ -944,23 +944,23 @@
           <t>Gross Revenue</t>
         </is>
       </c>
-      <c r="C19" s="12">
+      <c r="C19" s="13">
         <f>'5-Year Pro-Forma'!C24</f>
         <v/>
       </c>
-      <c r="D19" s="12">
+      <c r="D19" s="13">
         <f>'5-Year Pro-Forma'!D24</f>
         <v/>
       </c>
-      <c r="E19" s="12">
+      <c r="E19" s="13">
         <f>'5-Year Pro-Forma'!E24</f>
         <v/>
       </c>
-      <c r="F19" s="12">
+      <c r="F19" s="13">
         <f>'5-Year Pro-Forma'!F24</f>
         <v/>
       </c>
-      <c r="G19" s="12">
+      <c r="G19" s="13">
         <f>'5-Year Pro-Forma'!G24</f>
         <v/>
       </c>
@@ -971,50 +971,50 @@
           <t>Less: Upfront Prepay Discounts (15%)</t>
         </is>
       </c>
-      <c r="C20" s="12">
+      <c r="C20" s="13">
         <f>'5-Year Pro-Forma'!C25</f>
         <v/>
       </c>
-      <c r="D20" s="12">
+      <c r="D20" s="13">
         <f>'5-Year Pro-Forma'!D25</f>
         <v/>
       </c>
-      <c r="E20" s="12">
+      <c r="E20" s="13">
         <f>'5-Year Pro-Forma'!E25</f>
         <v/>
       </c>
-      <c r="F20" s="12">
+      <c r="F20" s="13">
         <f>'5-Year Pro-Forma'!F25</f>
         <v/>
       </c>
-      <c r="G20" s="12">
+      <c r="G20" s="13">
         <f>'5-Year Pro-Forma'!G25</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B21" s="14" t="inlineStr">
         <is>
           <t>Net Recognized Revenue</t>
         </is>
       </c>
-      <c r="C21" s="14">
+      <c r="C21" s="15">
         <f>'5-Year Pro-Forma'!C26</f>
         <v/>
       </c>
-      <c r="D21" s="14">
+      <c r="D21" s="15">
         <f>'5-Year Pro-Forma'!D26</f>
         <v/>
       </c>
-      <c r="E21" s="14">
+      <c r="E21" s="15">
         <f>'5-Year Pro-Forma'!E26</f>
         <v/>
       </c>
-      <c r="F21" s="14">
+      <c r="F21" s="15">
         <f>'5-Year Pro-Forma'!F26</f>
         <v/>
       </c>
-      <c r="G21" s="14">
+      <c r="G21" s="15">
         <f>'5-Year Pro-Forma'!G26</f>
         <v/>
       </c>
@@ -1026,50 +1026,50 @@
           <t>Cost of Goods Sold (COGS)</t>
         </is>
       </c>
-      <c r="C23" s="12">
+      <c r="C23" s="13">
         <f>'5-Year Pro-Forma'!C33</f>
         <v/>
       </c>
-      <c r="D23" s="12">
+      <c r="D23" s="13">
         <f>'5-Year Pro-Forma'!D33</f>
         <v/>
       </c>
-      <c r="E23" s="12">
+      <c r="E23" s="13">
         <f>'5-Year Pro-Forma'!E33</f>
         <v/>
       </c>
-      <c r="F23" s="12">
+      <c r="F23" s="13">
         <f>'5-Year Pro-Forma'!F33</f>
         <v/>
       </c>
-      <c r="G23" s="12">
+      <c r="G23" s="13">
         <f>'5-Year Pro-Forma'!G33</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="13" t="inlineStr">
+      <c r="B24" s="14" t="inlineStr">
         <is>
           <t>Gross Profit</t>
         </is>
       </c>
-      <c r="C24" s="15">
+      <c r="C24" s="16">
         <f>'5-Year Pro-Forma'!C34</f>
         <v/>
       </c>
-      <c r="D24" s="15">
+      <c r="D24" s="16">
         <f>'5-Year Pro-Forma'!D34</f>
         <v/>
       </c>
-      <c r="E24" s="15">
+      <c r="E24" s="16">
         <f>'5-Year Pro-Forma'!E34</f>
         <v/>
       </c>
-      <c r="F24" s="15">
+      <c r="F24" s="16">
         <f>'5-Year Pro-Forma'!F34</f>
         <v/>
       </c>
-      <c r="G24" s="15">
+      <c r="G24" s="16">
         <f>'5-Year Pro-Forma'!G34</f>
         <v/>
       </c>
@@ -1080,23 +1080,23 @@
           <t>Gross Margin %</t>
         </is>
       </c>
-      <c r="C25" s="16">
+      <c r="C25" s="17">
         <f>'5-Year Pro-Forma'!C35</f>
         <v/>
       </c>
-      <c r="D25" s="16">
+      <c r="D25" s="17">
         <f>'5-Year Pro-Forma'!D35</f>
         <v/>
       </c>
-      <c r="E25" s="16">
+      <c r="E25" s="17">
         <f>'5-Year Pro-Forma'!E35</f>
         <v/>
       </c>
-      <c r="F25" s="16">
+      <c r="F25" s="17">
         <f>'5-Year Pro-Forma'!F35</f>
         <v/>
       </c>
-      <c r="G25" s="16">
+      <c r="G25" s="17">
         <f>'5-Year Pro-Forma'!G35</f>
         <v/>
       </c>
@@ -1108,23 +1108,23 @@
           <t>Research &amp; Development (R&amp;D)</t>
         </is>
       </c>
-      <c r="C27" s="12">
+      <c r="C27" s="13">
         <f>'5-Year Pro-Forma'!C38</f>
         <v/>
       </c>
-      <c r="D27" s="12">
+      <c r="D27" s="13">
         <f>'5-Year Pro-Forma'!D38</f>
         <v/>
       </c>
-      <c r="E27" s="12">
+      <c r="E27" s="13">
         <f>'5-Year Pro-Forma'!E38</f>
         <v/>
       </c>
-      <c r="F27" s="12">
+      <c r="F27" s="13">
         <f>'5-Year Pro-Forma'!F38</f>
         <v/>
       </c>
-      <c r="G27" s="12">
+      <c r="G27" s="13">
         <f>'5-Year Pro-Forma'!G38</f>
         <v/>
       </c>
@@ -1135,23 +1135,23 @@
           <t>Sales &amp; Trading BD (S&amp;M)</t>
         </is>
       </c>
-      <c r="C28" s="12">
+      <c r="C28" s="13">
         <f>'5-Year Pro-Forma'!C39</f>
         <v/>
       </c>
-      <c r="D28" s="12">
+      <c r="D28" s="13">
         <f>'5-Year Pro-Forma'!D39</f>
         <v/>
       </c>
-      <c r="E28" s="12">
+      <c r="E28" s="13">
         <f>'5-Year Pro-Forma'!E39</f>
         <v/>
       </c>
-      <c r="F28" s="12">
+      <c r="F28" s="13">
         <f>'5-Year Pro-Forma'!F39</f>
         <v/>
       </c>
-      <c r="G28" s="12">
+      <c r="G28" s="13">
         <f>'5-Year Pro-Forma'!G39</f>
         <v/>
       </c>
@@ -1162,23 +1162,23 @@
           <t>General &amp; Administrative (G&amp;A)</t>
         </is>
       </c>
-      <c r="C29" s="12">
+      <c r="C29" s="13">
         <f>'5-Year Pro-Forma'!C40</f>
         <v/>
       </c>
-      <c r="D29" s="12">
+      <c r="D29" s="13">
         <f>'5-Year Pro-Forma'!D40</f>
         <v/>
       </c>
-      <c r="E29" s="12">
+      <c r="E29" s="13">
         <f>'5-Year Pro-Forma'!E40</f>
         <v/>
       </c>
-      <c r="F29" s="12">
+      <c r="F29" s="13">
         <f>'5-Year Pro-Forma'!F40</f>
         <v/>
       </c>
-      <c r="G29" s="12">
+      <c r="G29" s="13">
         <f>'5-Year Pro-Forma'!G40</f>
         <v/>
       </c>
@@ -1189,78 +1189,78 @@
           <t>Total Operating Expenses</t>
         </is>
       </c>
-      <c r="C30" s="12">
+      <c r="C30" s="13">
         <f>'5-Year Pro-Forma'!C42</f>
         <v/>
       </c>
-      <c r="D30" s="12">
+      <c r="D30" s="13">
         <f>'5-Year Pro-Forma'!D42</f>
         <v/>
       </c>
-      <c r="E30" s="12">
+      <c r="E30" s="13">
         <f>'5-Year Pro-Forma'!E42</f>
         <v/>
       </c>
-      <c r="F30" s="12">
+      <c r="F30" s="13">
         <f>'5-Year Pro-Forma'!F42</f>
         <v/>
       </c>
-      <c r="G30" s="12">
+      <c r="G30" s="13">
         <f>'5-Year Pro-Forma'!G42</f>
         <v/>
       </c>
     </row>
     <row r="31"/>
     <row r="32">
-      <c r="B32" s="13" t="inlineStr">
+      <c r="B32" s="14" t="inlineStr">
         <is>
           <t>EBITDA (Operating Profit)</t>
         </is>
       </c>
-      <c r="C32" s="15">
+      <c r="C32" s="16">
         <f>'5-Year Pro-Forma'!C45</f>
         <v/>
       </c>
-      <c r="D32" s="15">
+      <c r="D32" s="16">
         <f>'5-Year Pro-Forma'!D45</f>
         <v/>
       </c>
-      <c r="E32" s="15">
+      <c r="E32" s="16">
         <f>'5-Year Pro-Forma'!E45</f>
         <v/>
       </c>
-      <c r="F32" s="15">
+      <c r="F32" s="16">
         <f>'5-Year Pro-Forma'!F45</f>
         <v/>
       </c>
-      <c r="G32" s="15">
+      <c r="G32" s="16">
         <f>'5-Year Pro-Forma'!G45</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="13" t="inlineStr">
+      <c r="B33" s="14" t="inlineStr">
         <is>
           <t>EBITDA Margin %</t>
         </is>
       </c>
-      <c r="C33" s="17">
+      <c r="C33" s="18">
         <f>'5-Year Pro-Forma'!C46</f>
         <v/>
       </c>
-      <c r="D33" s="17">
+      <c r="D33" s="18">
         <f>'5-Year Pro-Forma'!D46</f>
         <v/>
       </c>
-      <c r="E33" s="17">
+      <c r="E33" s="18">
         <f>'5-Year Pro-Forma'!E46</f>
         <v/>
       </c>
-      <c r="F33" s="17">
+      <c r="F33" s="18">
         <f>'5-Year Pro-Forma'!F46</f>
         <v/>
       </c>
-      <c r="G33" s="17">
+      <c r="G33" s="18">
         <f>'5-Year Pro-Forma'!G46</f>
         <v/>
       </c>
@@ -1271,105 +1271,105 @@
           <t>Operating Income (EBIT)</t>
         </is>
       </c>
-      <c r="C34" s="12">
+      <c r="C34" s="13">
         <f>'5-Year Pro-Forma'!C48</f>
         <v/>
       </c>
-      <c r="D34" s="12">
+      <c r="D34" s="13">
         <f>'5-Year Pro-Forma'!D48</f>
         <v/>
       </c>
-      <c r="E34" s="12">
+      <c r="E34" s="13">
         <f>'5-Year Pro-Forma'!E48</f>
         <v/>
       </c>
-      <c r="F34" s="12">
+      <c r="F34" s="13">
         <f>'5-Year Pro-Forma'!F48</f>
         <v/>
       </c>
-      <c r="G34" s="12">
+      <c r="G34" s="13">
         <f>'5-Year Pro-Forma'!G48</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="13" t="inlineStr">
+      <c r="B35" s="14" t="inlineStr">
         <is>
           <t>Net Income (After Tax)</t>
         </is>
       </c>
-      <c r="C35" s="14">
+      <c r="C35" s="15">
         <f>'5-Year Pro-Forma'!C52</f>
         <v/>
       </c>
-      <c r="D35" s="14">
+      <c r="D35" s="15">
         <f>'5-Year Pro-Forma'!D52</f>
         <v/>
       </c>
-      <c r="E35" s="14">
+      <c r="E35" s="15">
         <f>'5-Year Pro-Forma'!E52</f>
         <v/>
       </c>
-      <c r="F35" s="14">
+      <c r="F35" s="15">
         <f>'5-Year Pro-Forma'!F52</f>
         <v/>
       </c>
-      <c r="G35" s="14">
+      <c r="G35" s="15">
         <f>'5-Year Pro-Forma'!G52</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="13" t="inlineStr">
+      <c r="B36" s="14" t="inlineStr">
         <is>
           <t>Net Income Margin %</t>
         </is>
       </c>
-      <c r="C36" s="18">
+      <c r="C36" s="19">
         <f>'5-Year Pro-Forma'!C53</f>
         <v/>
       </c>
-      <c r="D36" s="18">
+      <c r="D36" s="19">
         <f>'5-Year Pro-Forma'!D53</f>
         <v/>
       </c>
-      <c r="E36" s="18">
+      <c r="E36" s="19">
         <f>'5-Year Pro-Forma'!E53</f>
         <v/>
       </c>
-      <c r="F36" s="18">
+      <c r="F36" s="19">
         <f>'5-Year Pro-Forma'!F53</f>
         <v/>
       </c>
-      <c r="G36" s="18">
+      <c r="G36" s="19">
         <f>'5-Year Pro-Forma'!G53</f>
         <v/>
       </c>
     </row>
     <row r="37"/>
     <row r="38">
-      <c r="B38" s="13" t="inlineStr">
+      <c r="B38" s="14" t="inlineStr">
         <is>
           <t>Implied Valuation (25x ARR Multiple)</t>
         </is>
       </c>
-      <c r="C38" s="15">
+      <c r="C38" s="16">
         <f>'Valuation &amp; Returns'!C21</f>
         <v/>
       </c>
-      <c r="D38" s="15">
+      <c r="D38" s="16">
         <f>'Valuation &amp; Returns'!D21</f>
         <v/>
       </c>
-      <c r="E38" s="15">
+      <c r="E38" s="16">
         <f>'Valuation &amp; Returns'!E21</f>
         <v/>
       </c>
-      <c r="F38" s="15">
+      <c r="F38" s="16">
         <f>'Valuation &amp; Returns'!F21</f>
         <v/>
       </c>
-      <c r="G38" s="15">
+      <c r="G38" s="16">
         <f>'Valuation &amp; Returns'!G21</f>
         <v/>
       </c>
@@ -1449,15 +1449,15 @@
           <t>Total Global Event Derivatives Market Notional (Y1)</t>
         </is>
       </c>
-      <c r="C7" s="19" t="n">
+      <c r="C7" s="20" t="n">
         <v>12000</v>
       </c>
-      <c r="D7" s="20" t="inlineStr">
+      <c r="D7" s="21" t="inlineStr">
         <is>
           <t>$M</t>
         </is>
       </c>
-      <c r="E7" s="21" t="inlineStr">
+      <c r="E7" s="22" t="inlineStr">
         <is>
           <t>Estimated 2026 combined Polymarket + Kalshi + ForecastEx volume</t>
         </is>
@@ -1469,15 +1469,15 @@
           <t>Total Global Event Derivatives Market Notional (Y3)</t>
         </is>
       </c>
-      <c r="C8" s="19" t="n">
+      <c r="C8" s="20" t="n">
         <v>85000</v>
       </c>
-      <c r="D8" s="20" t="inlineStr">
+      <c r="D8" s="21" t="inlineStr">
         <is>
           <t>$M</t>
         </is>
       </c>
-      <c r="E8" s="21" t="inlineStr">
+      <c r="E8" s="22" t="inlineStr">
         <is>
           <t>Expansion into macro indices, rates, and corporate earnings</t>
         </is>
@@ -1489,15 +1489,15 @@
           <t>Total Global Event Derivatives Market Notional (Y5)</t>
         </is>
       </c>
-      <c r="C9" s="19" t="n">
+      <c r="C9" s="20" t="n">
         <v>320000</v>
       </c>
-      <c r="D9" s="20" t="inlineStr">
+      <c r="D9" s="21" t="inlineStr">
         <is>
           <t>$M</t>
         </is>
       </c>
-      <c r="E9" s="21" t="inlineStr">
+      <c r="E9" s="22" t="inlineStr">
         <is>
           <t>Institutional scale capturing 0.2% of global macro hedging</t>
         </is>
@@ -1509,15 +1509,15 @@
           <t>PRISM Share of Institutional Routed Flow (Y1)</t>
         </is>
       </c>
-      <c r="C10" s="22" t="n">
+      <c r="C10" s="23" t="n">
         <v>0.008</v>
       </c>
-      <c r="D10" s="20" t="inlineStr">
+      <c r="D10" s="21" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E10" s="21" t="inlineStr">
+      <c r="E10" s="22" t="inlineStr">
         <is>
           <t>Capturing 0.8% of market volume in Seed year ($96M/yr)</t>
         </is>
@@ -1529,15 +1529,15 @@
           <t>PRISM Share of Institutional Routed Flow (Y3)</t>
         </is>
       </c>
-      <c r="C11" s="22" t="n">
+      <c r="C11" s="23" t="n">
         <v>0.052</v>
       </c>
-      <c r="D11" s="20" t="inlineStr">
+      <c r="D11" s="21" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E11" s="21" t="inlineStr">
+      <c r="E11" s="22" t="inlineStr">
         <is>
           <t>Capturing 5.2% of total market volume ($4.42B/yr)</t>
         </is>
@@ -1549,15 +1549,15 @@
           <t>PRISM Share of Institutional Routed Flow (Y5)</t>
         </is>
       </c>
-      <c r="C12" s="22" t="n">
+      <c r="C12" s="23" t="n">
         <v>0.12</v>
       </c>
-      <c r="D12" s="20" t="inlineStr">
+      <c r="D12" s="21" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E12" s="21" t="inlineStr">
+      <c r="E12" s="22" t="inlineStr">
         <is>
           <t>Capturing 12.0% as category king execution standard ($38.4B/yr)</t>
         </is>
@@ -1599,15 +1599,15 @@
           <t>Tier 1: Core Quant API</t>
         </is>
       </c>
-      <c r="C16" s="23" t="n">
+      <c r="C16" s="24" t="n">
         <v>2500</v>
       </c>
-      <c r="D16" s="20" t="inlineStr">
+      <c r="D16" s="21" t="inlineStr">
         <is>
           <t>$</t>
         </is>
       </c>
-      <c r="E16" s="21" t="inlineStr">
+      <c r="E16" s="22" t="inlineStr">
         <is>
           <t>Systematic algo bots, 100 req/sec, standard REST/WebSocket</t>
         </is>
@@ -1619,15 +1619,15 @@
           <t>Tier 2: Institutional Desk (Core Flagship)</t>
         </is>
       </c>
-      <c r="C17" s="23" t="n">
+      <c r="C17" s="24" t="n">
         <v>12000</v>
       </c>
-      <c r="D17" s="20" t="inlineStr">
+      <c r="D17" s="21" t="inlineStr">
         <is>
           <t>$</t>
         </is>
       </c>
-      <c r="E17" s="21" t="inlineStr">
+      <c r="E17" s="22" t="inlineStr">
         <is>
           <t>Multi-seat terminal, Parity Radar, Oracle Conflict Guard, 99.95% SLA</t>
         </is>
@@ -1639,15 +1639,15 @@
           <t>Tier 3: Prime Direct (Enterprise)</t>
         </is>
       </c>
-      <c r="C18" s="23" t="n">
+      <c r="C18" s="24" t="n">
         <v>35000</v>
       </c>
-      <c r="D18" s="20" t="inlineStr">
+      <c r="D18" s="21" t="inlineStr">
         <is>
           <t>$</t>
         </is>
       </c>
-      <c r="E18" s="21" t="inlineStr">
+      <c r="E18" s="22" t="inlineStr">
         <is>
           <t>Dedicated VPC instance, custom Iceberg/TWAP algos, FIX drop-copy</t>
         </is>
@@ -1659,15 +1659,15 @@
           <t>Tier 4: Sovereign Co-Location (Secaucus NY4)</t>
         </is>
       </c>
-      <c r="C19" s="23" t="n">
+      <c r="C19" s="24" t="n">
         <v>65000</v>
       </c>
-      <c r="D19" s="20" t="inlineStr">
+      <c r="D19" s="21" t="inlineStr">
         <is>
           <t>$</t>
         </is>
       </c>
-      <c r="E19" s="21" t="inlineStr">
+      <c r="E19" s="22" t="inlineStr">
         <is>
           <t>Direct Equinix NY4 10Gbps cross-connect, sub-0.5ms FPGA path</t>
         </is>
@@ -1679,15 +1679,15 @@
           <t>Annual Upfront Prepay Discount</t>
         </is>
       </c>
-      <c r="C20" s="22" t="n">
+      <c r="C20" s="23" t="n">
         <v>0.15</v>
       </c>
-      <c r="D20" s="20" t="inlineStr">
+      <c r="D20" s="21" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E20" s="21" t="inlineStr">
+      <c r="E20" s="22" t="inlineStr">
         <is>
           <t>15% discount for 12-month upfront cash payment (creates negative working capital)</t>
         </is>
@@ -1699,15 +1699,15 @@
           <t>Expected % of Clients Choosing Annual Prepay</t>
         </is>
       </c>
-      <c r="C21" s="22" t="n">
+      <c r="C21" s="23" t="n">
         <v>0.45</v>
       </c>
-      <c r="D21" s="20" t="inlineStr">
+      <c r="D21" s="21" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E21" s="21" t="inlineStr">
+      <c r="E21" s="22" t="inlineStr">
         <is>
           <t>Funds taking advantage of annual budget allocation discounts</t>
         </is>
@@ -1749,15 +1749,15 @@
           <t>Standard Volume Routing Take-Rate</t>
         </is>
       </c>
-      <c r="C25" s="22" t="n">
+      <c r="C25" s="23" t="n">
         <v>0.00015</v>
       </c>
-      <c r="D25" s="20" t="inlineStr">
+      <c r="D25" s="21" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E25" s="21" t="inlineStr">
+      <c r="E25" s="22" t="inlineStr">
         <is>
           <t>1.5 bps (0.015%) charged on net notional executed through SOR</t>
         </is>
@@ -1769,15 +1769,15 @@
           <t>Average Slippage Saved per Client Order</t>
         </is>
       </c>
-      <c r="C26" s="22" t="n">
+      <c r="C26" s="23" t="n">
         <v>0.0296</v>
       </c>
-      <c r="D26" s="20" t="inlineStr">
+      <c r="D26" s="21" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E26" s="21" t="inlineStr">
+      <c r="E26" s="22" t="inlineStr">
         <is>
           <t>296 bps saved vs single-venue execution (clients retain 95% of alpha)</t>
         </is>
@@ -1789,15 +1789,15 @@
           <t>Client Value-to-Fee Ratio</t>
         </is>
       </c>
-      <c r="C27" s="24" t="n">
+      <c r="C27" s="25" t="n">
         <v>19.7</v>
       </c>
-      <c r="D27" s="20" t="inlineStr">
+      <c r="D27" s="21" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="E27" s="21" t="inlineStr">
+      <c r="E27" s="22" t="inlineStr">
         <is>
           <t>Clients save $19.70 for every $1.00 paid to PRISM in routing fees</t>
         </is>
@@ -1839,15 +1839,15 @@
           <t>Tier 2 CAC (Institutional Desk)</t>
         </is>
       </c>
-      <c r="C31" s="23" t="n">
+      <c r="C31" s="24" t="n">
         <v>22000</v>
       </c>
-      <c r="D31" s="20" t="inlineStr">
+      <c r="D31" s="21" t="inlineStr">
         <is>
           <t>$</t>
         </is>
       </c>
-      <c r="E31" s="21" t="inlineStr">
+      <c r="E31" s="22" t="inlineStr">
         <is>
           <t>Technical sales engineer salary, compliance review, POC demo period</t>
         </is>
@@ -1859,15 +1859,15 @@
           <t>Tier 3 CAC (Prime Direct)</t>
         </is>
       </c>
-      <c r="C32" s="23" t="n">
+      <c r="C32" s="24" t="n">
         <v>65000</v>
       </c>
-      <c r="D32" s="20" t="inlineStr">
+      <c r="D32" s="21" t="inlineStr">
         <is>
           <t>$</t>
         </is>
       </c>
-      <c r="E32" s="21" t="inlineStr">
+      <c r="E32" s="22" t="inlineStr">
         <is>
           <t>Enterprise procurement, on-premise security review, legal review</t>
         </is>
@@ -1879,15 +1879,15 @@
           <t>Sales Cycle Duration (Tier 2)</t>
         </is>
       </c>
-      <c r="C33" s="19" t="n">
+      <c r="C33" s="20" t="n">
         <v>45</v>
       </c>
-      <c r="D33" s="20" t="inlineStr">
+      <c r="D33" s="21" t="inlineStr">
         <is>
           <t>Days</t>
         </is>
       </c>
-      <c r="E33" s="21" t="inlineStr">
+      <c r="E33" s="22" t="inlineStr">
         <is>
           <t>Rapid trial-to-production deployment timeline</t>
         </is>
@@ -1899,15 +1899,15 @@
           <t>Annual Gross Logo Churn Rate</t>
         </is>
       </c>
-      <c r="C34" s="22" t="n">
+      <c r="C34" s="23" t="n">
         <v>0.05</v>
       </c>
-      <c r="D34" s="20" t="inlineStr">
+      <c r="D34" s="21" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E34" s="21" t="inlineStr">
+      <c r="E34" s="22" t="inlineStr">
         <is>
           <t>5% annual churn (OEMS workflow integration creates high stickiness)</t>
         </is>
@@ -1919,15 +1919,15 @@
           <t>Net Revenue Retention (NRR)</t>
         </is>
       </c>
-      <c r="C35" s="22" t="n">
+      <c r="C35" s="23" t="n">
         <v>1.28</v>
       </c>
-      <c r="D35" s="20" t="inlineStr">
+      <c r="D35" s="21" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E35" s="21" t="inlineStr">
+      <c r="E35" s="22" t="inlineStr">
         <is>
           <t>128% NRR driven by funds adding seats and increasing routed volume</t>
         </is>
@@ -1969,15 +1969,15 @@
           <t>Equinix NY4 Secaucus Cabinet Base Lease</t>
         </is>
       </c>
-      <c r="C39" s="23" t="n">
+      <c r="C39" s="24" t="n">
         <v>6500</v>
       </c>
-      <c r="D39" s="20" t="inlineStr">
+      <c r="D39" s="21" t="inlineStr">
         <is>
           <t>$</t>
         </is>
       </c>
-      <c r="E39" s="21" t="inlineStr">
+      <c r="E39" s="22" t="inlineStr">
         <is>
           <t>1U-4U rack space, redundant PDU, Secaucus datacenter</t>
         </is>
@@ -1989,15 +1989,15 @@
           <t>NY4 Cross-Connect per 10 Active Clients</t>
         </is>
       </c>
-      <c r="C40" s="23" t="n">
+      <c r="C40" s="24" t="n">
         <v>1200</v>
       </c>
-      <c r="D40" s="20" t="inlineStr">
+      <c r="D40" s="21" t="inlineStr">
         <is>
           <t>$</t>
         </is>
       </c>
-      <c r="E40" s="21" t="inlineStr">
+      <c r="E40" s="22" t="inlineStr">
         <is>
           <t>Direct low-latency fiber cross-connects to exchange matching engines</t>
         </is>
@@ -2009,15 +2009,15 @@
           <t>Enterprise L2 RPC Nodes (Polygon/Arbitrum)</t>
         </is>
       </c>
-      <c r="C41" s="23" t="n">
+      <c r="C41" s="24" t="n">
         <v>2200</v>
       </c>
-      <c r="D41" s="20" t="inlineStr">
+      <c r="D41" s="21" t="inlineStr">
         <is>
           <t>$</t>
         </is>
       </c>
-      <c r="E41" s="21" t="inlineStr">
+      <c r="E41" s="22" t="inlineStr">
         <is>
           <t>Dedicated high-throughput Alchemy/QuickNode endpoints</t>
         </is>
@@ -2029,15 +2029,15 @@
           <t>AWS/GCP Serverless Engine Base</t>
         </is>
       </c>
-      <c r="C42" s="23" t="n">
+      <c r="C42" s="24" t="n">
         <v>1800</v>
       </c>
-      <c r="D42" s="20" t="inlineStr">
+      <c r="D42" s="21" t="inlineStr">
         <is>
           <t>$</t>
         </is>
       </c>
-      <c r="E42" s="21" t="inlineStr">
+      <c r="E42" s="22" t="inlineStr">
         <is>
           <t>Database clusters, Redis low-latency cache, API gateways</t>
         </is>
@@ -2049,15 +2049,15 @@
           <t>Cloud Variable Cost per $1M Routed</t>
         </is>
       </c>
-      <c r="C43" s="23" t="n">
+      <c r="C43" s="24" t="n">
         <v>12</v>
       </c>
-      <c r="D43" s="20" t="inlineStr">
+      <c r="D43" s="21" t="inlineStr">
         <is>
           <t>$</t>
         </is>
       </c>
-      <c r="E43" s="21" t="inlineStr">
+      <c r="E43" s="22" t="inlineStr">
         <is>
           <t>Elastic serverless execution scaling per order million</t>
         </is>
@@ -2069,15 +2069,15 @@
           <t>FIPS 140-2 Level 3 HSM Hardware Security</t>
         </is>
       </c>
-      <c r="C44" s="23" t="n">
+      <c r="C44" s="24" t="n">
         <v>1500</v>
       </c>
-      <c r="D44" s="20" t="inlineStr">
+      <c r="D44" s="21" t="inlineStr">
         <is>
           <t>$</t>
         </is>
       </c>
-      <c r="E44" s="21" t="inlineStr">
+      <c r="E44" s="22" t="inlineStr">
         <is>
           <t>Dedicated cryptographic key validation hardware</t>
         </is>
@@ -2089,15 +2089,15 @@
           <t>Real-Time L2 Market Data Streaming Relays</t>
         </is>
       </c>
-      <c r="C45" s="23" t="n">
+      <c r="C45" s="24" t="n">
         <v>2000</v>
       </c>
-      <c r="D45" s="20" t="inlineStr">
+      <c r="D45" s="21" t="inlineStr">
         <is>
           <t>$</t>
         </is>
       </c>
-      <c r="E45" s="21" t="inlineStr">
+      <c r="E45" s="22" t="inlineStr">
         <is>
           <t>WebSocket distribution clusters</t>
         </is>
@@ -2139,15 +2139,15 @@
           <t>Low-Latency / C++ / Rust Systems Engineer</t>
         </is>
       </c>
-      <c r="C49" s="23" t="n">
+      <c r="C49" s="24" t="n">
         <v>210000</v>
       </c>
-      <c r="D49" s="20" t="inlineStr">
+      <c r="D49" s="21" t="inlineStr">
         <is>
           <t>$</t>
         </is>
       </c>
-      <c r="E49" s="21" t="inlineStr">
+      <c r="E49" s="22" t="inlineStr">
         <is>
           <t>$256,200 fully loaded annual compensation</t>
         </is>
@@ -2159,15 +2159,15 @@
           <t>Quantitative Microstructure Researcher</t>
         </is>
       </c>
-      <c r="C50" s="23" t="n">
+      <c r="C50" s="24" t="n">
         <v>220000</v>
       </c>
-      <c r="D50" s="20" t="inlineStr">
+      <c r="D50" s="21" t="inlineStr">
         <is>
           <t>$</t>
         </is>
       </c>
-      <c r="E50" s="21" t="inlineStr">
+      <c r="E50" s="22" t="inlineStr">
         <is>
           <t>$268,400 fully loaded annual compensation</t>
         </is>
@@ -2179,15 +2179,15 @@
           <t>VP Institutional Sales / Business Dev</t>
         </is>
       </c>
-      <c r="C51" s="23" t="n">
+      <c r="C51" s="24" t="n">
         <v>160000</v>
       </c>
-      <c r="D51" s="20" t="inlineStr">
+      <c r="D51" s="21" t="inlineStr">
         <is>
           <t>$</t>
         </is>
       </c>
-      <c r="E51" s="21" t="inlineStr">
+      <c r="E51" s="22" t="inlineStr">
         <is>
           <t>$195,200 base + commission tied to desk quota</t>
         </is>
@@ -2199,15 +2199,15 @@
           <t>Solutions Architect / Desk Integration Engineer</t>
         </is>
       </c>
-      <c r="C52" s="23" t="n">
+      <c r="C52" s="24" t="n">
         <v>150000</v>
       </c>
-      <c r="D52" s="20" t="inlineStr">
+      <c r="D52" s="21" t="inlineStr">
         <is>
           <t>$</t>
         </is>
       </c>
-      <c r="E52" s="21" t="inlineStr">
+      <c r="E52" s="22" t="inlineStr">
         <is>
           <t>$183,000 fully loaded annual compensation</t>
         </is>
@@ -2219,15 +2219,15 @@
           <t>General Counsel &amp; Chief Compliance Officer</t>
         </is>
       </c>
-      <c r="C53" s="23" t="n">
+      <c r="C53" s="24" t="n">
         <v>200000</v>
       </c>
-      <c r="D53" s="20" t="inlineStr">
+      <c r="D53" s="21" t="inlineStr">
         <is>
           <t>$</t>
         </is>
       </c>
-      <c r="E53" s="21" t="inlineStr">
+      <c r="E53" s="22" t="inlineStr">
         <is>
           <t>$244,000 fully loaded annual compensation</t>
         </is>
@@ -2239,15 +2239,15 @@
           <t>Operations / Financial Controller</t>
         </is>
       </c>
-      <c r="C54" s="23" t="n">
+      <c r="C54" s="24" t="n">
         <v>140000</v>
       </c>
-      <c r="D54" s="20" t="inlineStr">
+      <c r="D54" s="21" t="inlineStr">
         <is>
           <t>$</t>
         </is>
       </c>
-      <c r="E54" s="21" t="inlineStr">
+      <c r="E54" s="22" t="inlineStr">
         <is>
           <t>$170,800 fully loaded annual compensation</t>
         </is>
@@ -2429,28 +2429,28 @@
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="14" t="inlineStr">
         <is>
           <t>Total Active Institutional Desks</t>
         </is>
       </c>
-      <c r="C12" s="25">
+      <c r="C12" s="26">
         <f>SUM(C8:C11)</f>
         <v/>
       </c>
-      <c r="D12" s="25">
+      <c r="D12" s="26">
         <f>SUM(D8:D11)</f>
         <v/>
       </c>
-      <c r="E12" s="25">
+      <c r="E12" s="26">
         <f>SUM(E8:E11)</f>
         <v/>
       </c>
-      <c r="F12" s="25">
+      <c r="F12" s="26">
         <f>SUM(F8:F11)</f>
         <v/>
       </c>
-      <c r="G12" s="25">
+      <c r="G12" s="26">
         <f>SUM(G8:G11)</f>
         <v/>
       </c>
@@ -2461,45 +2461,45 @@
           <t>Average Monthly Routed Volume per Desk ($M)</t>
         </is>
       </c>
-      <c r="C13" s="26" t="n">
+      <c r="C13" s="12" t="n">
         <v>6.7</v>
       </c>
-      <c r="D13" s="26" t="n">
+      <c r="D13" s="12" t="n">
         <v>7.3</v>
       </c>
-      <c r="E13" s="26" t="n">
+      <c r="E13" s="12" t="n">
         <v>10.8</v>
       </c>
-      <c r="F13" s="26" t="n">
+      <c r="F13" s="12" t="n">
         <v>14.2</v>
       </c>
-      <c r="G13" s="26" t="n">
+      <c r="G13" s="12" t="n">
         <v>17.5</v>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B14" s="14" t="inlineStr">
         <is>
           <t>Annual Routed Notional Volume ($M)</t>
         </is>
       </c>
-      <c r="C14" s="14">
+      <c r="C14" s="15">
         <f>C12*C13*12</f>
         <v/>
       </c>
-      <c r="D14" s="14">
+      <c r="D14" s="15">
         <f>D12*D13*12</f>
         <v/>
       </c>
-      <c r="E14" s="14">
+      <c r="E14" s="15">
         <f>E12*E13*12</f>
         <v/>
       </c>
-      <c r="F14" s="14">
+      <c r="F14" s="15">
         <f>F12*F13*12</f>
         <v/>
       </c>
-      <c r="G14" s="14">
+      <c r="G14" s="15">
         <f>G12*G13*12</f>
         <v/>
       </c>
@@ -2518,24 +2518,24 @@
           <t>Tier 1: Core Quant API Revenue</t>
         </is>
       </c>
-      <c r="C17" s="12">
-        <f>C8*'Model Assumptions'!C15*12</f>
-        <v/>
-      </c>
-      <c r="D17" s="12">
-        <f>D8*'Model Assumptions'!C15*12</f>
-        <v/>
-      </c>
-      <c r="E17" s="12">
-        <f>E8*'Model Assumptions'!C15*12</f>
-        <v/>
-      </c>
-      <c r="F17" s="12">
-        <f>F8*'Model Assumptions'!C15*12</f>
-        <v/>
-      </c>
-      <c r="G17" s="12">
-        <f>G8*'Model Assumptions'!C15*12</f>
+      <c r="C17" s="13">
+        <f>C8*'Model Assumptions'!C16*12</f>
+        <v/>
+      </c>
+      <c r="D17" s="13">
+        <f>D8*'Model Assumptions'!C16*12</f>
+        <v/>
+      </c>
+      <c r="E17" s="13">
+        <f>E8*'Model Assumptions'!C16*12</f>
+        <v/>
+      </c>
+      <c r="F17" s="13">
+        <f>F8*'Model Assumptions'!C16*12</f>
+        <v/>
+      </c>
+      <c r="G17" s="13">
+        <f>G8*'Model Assumptions'!C16*12</f>
         <v/>
       </c>
     </row>
@@ -2545,24 +2545,24 @@
           <t>Tier 2: Institutional Desk Revenue</t>
         </is>
       </c>
-      <c r="C18" s="12">
-        <f>C9*'Model Assumptions'!C16*12</f>
-        <v/>
-      </c>
-      <c r="D18" s="12">
-        <f>D9*'Model Assumptions'!C16*12</f>
-        <v/>
-      </c>
-      <c r="E18" s="12">
-        <f>E9*'Model Assumptions'!C16*12</f>
-        <v/>
-      </c>
-      <c r="F18" s="12">
-        <f>F9*'Model Assumptions'!C16*12</f>
-        <v/>
-      </c>
-      <c r="G18" s="12">
-        <f>G9*'Model Assumptions'!C16*12</f>
+      <c r="C18" s="13">
+        <f>C9*'Model Assumptions'!C17*12</f>
+        <v/>
+      </c>
+      <c r="D18" s="13">
+        <f>D9*'Model Assumptions'!C17*12</f>
+        <v/>
+      </c>
+      <c r="E18" s="13">
+        <f>E9*'Model Assumptions'!C17*12</f>
+        <v/>
+      </c>
+      <c r="F18" s="13">
+        <f>F9*'Model Assumptions'!C17*12</f>
+        <v/>
+      </c>
+      <c r="G18" s="13">
+        <f>G9*'Model Assumptions'!C17*12</f>
         <v/>
       </c>
     </row>
@@ -2572,24 +2572,24 @@
           <t>Tier 3: Prime Direct Revenue</t>
         </is>
       </c>
-      <c r="C19" s="12">
-        <f>C10*'Model Assumptions'!C17*12</f>
-        <v/>
-      </c>
-      <c r="D19" s="12">
-        <f>D10*'Model Assumptions'!C17*12</f>
-        <v/>
-      </c>
-      <c r="E19" s="12">
-        <f>E10*'Model Assumptions'!C17*12</f>
-        <v/>
-      </c>
-      <c r="F19" s="12">
-        <f>F10*'Model Assumptions'!C17*12</f>
-        <v/>
-      </c>
-      <c r="G19" s="12">
-        <f>G10*'Model Assumptions'!C17*12</f>
+      <c r="C19" s="13">
+        <f>C10*'Model Assumptions'!C18*12</f>
+        <v/>
+      </c>
+      <c r="D19" s="13">
+        <f>D10*'Model Assumptions'!C18*12</f>
+        <v/>
+      </c>
+      <c r="E19" s="13">
+        <f>E10*'Model Assumptions'!C18*12</f>
+        <v/>
+      </c>
+      <c r="F19" s="13">
+        <f>F10*'Model Assumptions'!C18*12</f>
+        <v/>
+      </c>
+      <c r="G19" s="13">
+        <f>G10*'Model Assumptions'!C18*12</f>
         <v/>
       </c>
     </row>
@@ -2599,29 +2599,29 @@
           <t>Tier 4: Sovereign Co-Lo Revenue</t>
         </is>
       </c>
-      <c r="C20" s="12">
-        <f>C11*'Model Assumptions'!C18*12</f>
-        <v/>
-      </c>
-      <c r="D20" s="12">
-        <f>D11*'Model Assumptions'!C18*12</f>
-        <v/>
-      </c>
-      <c r="E20" s="12">
-        <f>E11*'Model Assumptions'!C18*12</f>
-        <v/>
-      </c>
-      <c r="F20" s="12">
-        <f>F11*'Model Assumptions'!C18*12</f>
-        <v/>
-      </c>
-      <c r="G20" s="12">
-        <f>G11*'Model Assumptions'!C18*12</f>
+      <c r="C20" s="13">
+        <f>C11*'Model Assumptions'!C19*12</f>
+        <v/>
+      </c>
+      <c r="D20" s="13">
+        <f>D11*'Model Assumptions'!C19*12</f>
+        <v/>
+      </c>
+      <c r="E20" s="13">
+        <f>E11*'Model Assumptions'!C19*12</f>
+        <v/>
+      </c>
+      <c r="F20" s="13">
+        <f>F11*'Model Assumptions'!C19*12</f>
+        <v/>
+      </c>
+      <c r="G20" s="13">
+        <f>G11*'Model Assumptions'!C19*12</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B21" s="14" t="inlineStr">
         <is>
           <t>Total SaaS Subscription Revenue (ARR)</t>
         </is>
@@ -2653,24 +2653,24 @@
           <t>Volume Routing Take-Rate (1.5 bps)</t>
         </is>
       </c>
-      <c r="C22" s="12">
-        <f>C14*1000000*'Model Assumptions'!C24</f>
-        <v/>
-      </c>
-      <c r="D22" s="12">
-        <f>D14*1000000*'Model Assumptions'!C24</f>
-        <v/>
-      </c>
-      <c r="E22" s="12">
-        <f>E14*1000000*'Model Assumptions'!C24</f>
-        <v/>
-      </c>
-      <c r="F22" s="12">
-        <f>F14*1000000*'Model Assumptions'!C24</f>
-        <v/>
-      </c>
-      <c r="G22" s="12">
-        <f>G14*1000000*'Model Assumptions'!C24</f>
+      <c r="C22" s="13">
+        <f>C14*1000000*'Model Assumptions'!C25</f>
+        <v/>
+      </c>
+      <c r="D22" s="13">
+        <f>D14*1000000*'Model Assumptions'!C25</f>
+        <v/>
+      </c>
+      <c r="E22" s="13">
+        <f>E14*1000000*'Model Assumptions'!C25</f>
+        <v/>
+      </c>
+      <c r="F22" s="13">
+        <f>F14*1000000*'Model Assumptions'!C25</f>
+        <v/>
+      </c>
+      <c r="G22" s="13">
+        <f>G14*1000000*'Model Assumptions'!C25</f>
         <v/>
       </c>
     </row>
@@ -2680,24 +2680,24 @@
           <t>Premium Data &amp; Legal Oracle Feeds</t>
         </is>
       </c>
-      <c r="C23" s="12" t="n">
+      <c r="C23" s="13" t="n">
         <v>75000</v>
       </c>
-      <c r="D23" s="12" t="n">
+      <c r="D23" s="13" t="n">
         <v>360000</v>
       </c>
-      <c r="E23" s="12" t="n">
+      <c r="E23" s="13" t="n">
         <v>1100000</v>
       </c>
-      <c r="F23" s="12" t="n">
+      <c r="F23" s="13" t="n">
         <v>2400000</v>
       </c>
-      <c r="G23" s="12" t="n">
+      <c r="G23" s="13" t="n">
         <v>4200000</v>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="13" t="inlineStr">
+      <c r="B24" s="14" t="inlineStr">
         <is>
           <t>Total Gross Contracted Revenue</t>
         </is>
@@ -2729,29 +2729,29 @@
           <t>Less: Annual Prepay Cash Discounts</t>
         </is>
       </c>
-      <c r="C25" s="12">
-        <f>-C21*'Model Assumptions'!C19*'Model Assumptions'!C20</f>
-        <v/>
-      </c>
-      <c r="D25" s="12">
-        <f>-D21*'Model Assumptions'!C19*'Model Assumptions'!C20</f>
-        <v/>
-      </c>
-      <c r="E25" s="12">
-        <f>-E21*'Model Assumptions'!C19*'Model Assumptions'!C20</f>
-        <v/>
-      </c>
-      <c r="F25" s="12">
-        <f>-F21*'Model Assumptions'!C19*'Model Assumptions'!C20</f>
-        <v/>
-      </c>
-      <c r="G25" s="12">
-        <f>-G21*'Model Assumptions'!C19*'Model Assumptions'!C20</f>
+      <c r="C25" s="13">
+        <f>-C21*'Model Assumptions'!C20*'Model Assumptions'!C21</f>
+        <v/>
+      </c>
+      <c r="D25" s="13">
+        <f>-D21*'Model Assumptions'!C20*'Model Assumptions'!C21</f>
+        <v/>
+      </c>
+      <c r="E25" s="13">
+        <f>-E21*'Model Assumptions'!C20*'Model Assumptions'!C21</f>
+        <v/>
+      </c>
+      <c r="F25" s="13">
+        <f>-F21*'Model Assumptions'!C20*'Model Assumptions'!C21</f>
+        <v/>
+      </c>
+      <c r="G25" s="13">
+        <f>-G21*'Model Assumptions'!C20*'Model Assumptions'!C21</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="13" t="inlineStr">
+      <c r="B26" s="14" t="inlineStr">
         <is>
           <t>NET RECOGNIZED REVENUE</t>
         </is>
@@ -2791,24 +2791,24 @@
           <t>Equinix NY4 Co-Location &amp; Cross-Connects</t>
         </is>
       </c>
-      <c r="C29" s="12">
-        <f>('Model Assumptions'!C36*12)+(C12*'Model Assumptions'!C37*12/10)</f>
-        <v/>
-      </c>
-      <c r="D29" s="12">
-        <f>('Model Assumptions'!C36*12)+(D12*'Model Assumptions'!C37*12/10)</f>
-        <v/>
-      </c>
-      <c r="E29" s="12">
-        <f>('Model Assumptions'!C36*12)+(E12*'Model Assumptions'!C37*12/10)</f>
-        <v/>
-      </c>
-      <c r="F29" s="12">
-        <f>('Model Assumptions'!C36*12)+(F12*'Model Assumptions'!C37*12/10)</f>
-        <v/>
-      </c>
-      <c r="G29" s="12">
-        <f>('Model Assumptions'!C36*12)+(G12*'Model Assumptions'!C37*12/10)</f>
+      <c r="C29" s="13">
+        <f>('Model Assumptions'!C39*12)+(C12*'Model Assumptions'!C40*12/10)</f>
+        <v/>
+      </c>
+      <c r="D29" s="13">
+        <f>('Model Assumptions'!C39*12)+(D12*'Model Assumptions'!C40*12/10)</f>
+        <v/>
+      </c>
+      <c r="E29" s="13">
+        <f>('Model Assumptions'!C39*12)+(E12*'Model Assumptions'!C40*12/10)</f>
+        <v/>
+      </c>
+      <c r="F29" s="13">
+        <f>('Model Assumptions'!C39*12)+(F12*'Model Assumptions'!C40*12/10)</f>
+        <v/>
+      </c>
+      <c r="G29" s="13">
+        <f>('Model Assumptions'!C39*12)+(G12*'Model Assumptions'!C40*12/10)</f>
         <v/>
       </c>
     </row>
@@ -2818,24 +2818,24 @@
           <t>Enterprise RPC Nodes &amp; L2 Gas Relayers</t>
         </is>
       </c>
-      <c r="C30" s="12">
-        <f>'Model Assumptions'!C38*12</f>
-        <v/>
-      </c>
-      <c r="D30" s="12">
-        <f>'Model Assumptions'!C38*12*1.8</f>
-        <v/>
-      </c>
-      <c r="E30" s="12">
-        <f>'Model Assumptions'!C38*12*3.2</f>
-        <v/>
-      </c>
-      <c r="F30" s="12">
-        <f>'Model Assumptions'!C38*12*5.5</f>
-        <v/>
-      </c>
-      <c r="G30" s="12">
-        <f>'Model Assumptions'!C38*12*8.0</f>
+      <c r="C30" s="13">
+        <f>'Model Assumptions'!C41*12</f>
+        <v/>
+      </c>
+      <c r="D30" s="13">
+        <f>'Model Assumptions'!C41*12*1.8</f>
+        <v/>
+      </c>
+      <c r="E30" s="13">
+        <f>'Model Assumptions'!C41*12*3.2</f>
+        <v/>
+      </c>
+      <c r="F30" s="13">
+        <f>'Model Assumptions'!C41*12*5.5</f>
+        <v/>
+      </c>
+      <c r="G30" s="13">
+        <f>'Model Assumptions'!C41*12*8.0</f>
         <v/>
       </c>
     </row>
@@ -2845,24 +2845,24 @@
           <t>Cloud Compute, Redis &amp; WebSocket Relays</t>
         </is>
       </c>
-      <c r="C31" s="12">
-        <f>('Model Assumptions'!C39*12)+(C14*'Model Assumptions'!C40)</f>
-        <v/>
-      </c>
-      <c r="D31" s="12">
-        <f>('Model Assumptions'!C39*12)+(D14*'Model Assumptions'!C40)</f>
-        <v/>
-      </c>
-      <c r="E31" s="12">
-        <f>('Model Assumptions'!C39*12)+(E14*'Model Assumptions'!C40)</f>
-        <v/>
-      </c>
-      <c r="F31" s="12">
-        <f>('Model Assumptions'!C39*12)+(F14*'Model Assumptions'!C40)</f>
-        <v/>
-      </c>
-      <c r="G31" s="12">
-        <f>('Model Assumptions'!C39*12)+(G14*'Model Assumptions'!C40)</f>
+      <c r="C31" s="13">
+        <f>('Model Assumptions'!C42*12)+(C14*'Model Assumptions'!C43)</f>
+        <v/>
+      </c>
+      <c r="D31" s="13">
+        <f>('Model Assumptions'!C42*12)+(D14*'Model Assumptions'!C43)</f>
+        <v/>
+      </c>
+      <c r="E31" s="13">
+        <f>('Model Assumptions'!C42*12)+(E14*'Model Assumptions'!C43)</f>
+        <v/>
+      </c>
+      <c r="F31" s="13">
+        <f>('Model Assumptions'!C42*12)+(F14*'Model Assumptions'!C43)</f>
+        <v/>
+      </c>
+      <c r="G31" s="13">
+        <f>('Model Assumptions'!C42*12)+(G14*'Model Assumptions'!C43)</f>
         <v/>
       </c>
     </row>
@@ -2872,29 +2872,29 @@
           <t>FIPS 140-2 Hardware HSM Cryptographic Security</t>
         </is>
       </c>
-      <c r="C32" s="12">
-        <f>'Model Assumptions'!C41*12</f>
-        <v/>
-      </c>
-      <c r="D32" s="12">
-        <f>'Model Assumptions'!C41*12*1.5</f>
-        <v/>
-      </c>
-      <c r="E32" s="12">
-        <f>'Model Assumptions'!C41*12*2.2</f>
-        <v/>
-      </c>
-      <c r="F32" s="12">
-        <f>'Model Assumptions'!C41*12*3.5</f>
-        <v/>
-      </c>
-      <c r="G32" s="12">
-        <f>'Model Assumptions'!C41*12*5.0</f>
+      <c r="C32" s="13">
+        <f>'Model Assumptions'!C44*12</f>
+        <v/>
+      </c>
+      <c r="D32" s="13">
+        <f>'Model Assumptions'!C44*12*1.5</f>
+        <v/>
+      </c>
+      <c r="E32" s="13">
+        <f>'Model Assumptions'!C44*12*2.2</f>
+        <v/>
+      </c>
+      <c r="F32" s="13">
+        <f>'Model Assumptions'!C44*12*3.5</f>
+        <v/>
+      </c>
+      <c r="G32" s="13">
+        <f>'Model Assumptions'!C44*12*5.0</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="13" t="inlineStr">
+      <c r="B33" s="14" t="inlineStr">
         <is>
           <t>TOTAL COST OF GOODS SOLD</t>
         </is>
@@ -2921,7 +2921,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="13" t="inlineStr">
+      <c r="B34" s="14" t="inlineStr">
         <is>
           <t>GROSS PROFIT</t>
         </is>
@@ -2953,23 +2953,23 @@
           <t>Gross Margin %</t>
         </is>
       </c>
-      <c r="C35" s="16">
+      <c r="C35" s="17">
         <f>C34/C26</f>
         <v/>
       </c>
-      <c r="D35" s="16">
+      <c r="D35" s="17">
         <f>D34/D26</f>
         <v/>
       </c>
-      <c r="E35" s="16">
+      <c r="E35" s="17">
         <f>E34/E26</f>
         <v/>
       </c>
-      <c r="F35" s="16">
+      <c r="F35" s="17">
         <f>F34/F26</f>
         <v/>
       </c>
-      <c r="G35" s="16">
+      <c r="G35" s="17">
         <f>G34/G26</f>
         <v/>
       </c>
@@ -2988,19 +2988,19 @@
           <t>Research &amp; Development (R&amp;D / Low-Latency Engineering)</t>
         </is>
       </c>
-      <c r="C38" s="12" t="n">
+      <c r="C38" s="13" t="n">
         <v>850000</v>
       </c>
-      <c r="D38" s="12" t="n">
+      <c r="D38" s="13" t="n">
         <v>1800000</v>
       </c>
-      <c r="E38" s="12" t="n">
+      <c r="E38" s="13" t="n">
         <v>3600000</v>
       </c>
-      <c r="F38" s="12" t="n">
+      <c r="F38" s="13" t="n">
         <v>6200000</v>
       </c>
-      <c r="G38" s="12" t="n">
+      <c r="G38" s="13" t="n">
         <v>9500000</v>
       </c>
     </row>
@@ -3010,19 +3010,19 @@
           <t>Sales &amp; Marketing (Institutional Sales, Travel, Marketing)</t>
         </is>
       </c>
-      <c r="C39" s="12" t="n">
+      <c r="C39" s="13" t="n">
         <v>220000</v>
       </c>
-      <c r="D39" s="12" t="n">
+      <c r="D39" s="13" t="n">
         <v>650000</v>
       </c>
-      <c r="E39" s="12" t="n">
+      <c r="E39" s="13" t="n">
         <v>1400000</v>
       </c>
-      <c r="F39" s="12" t="n">
+      <c r="F39" s="13" t="n">
         <v>2800000</v>
       </c>
-      <c r="G39" s="12" t="n">
+      <c r="G39" s="13" t="n">
         <v>4800000</v>
       </c>
     </row>
@@ -3032,19 +3032,19 @@
           <t>General &amp; Administrative (Legal, Compliance, Audits, Insurance)</t>
         </is>
       </c>
-      <c r="C40" s="12" t="n">
+      <c r="C40" s="13" t="n">
         <v>110000</v>
       </c>
-      <c r="D40" s="12" t="n">
+      <c r="D40" s="13" t="n">
         <v>240000</v>
       </c>
-      <c r="E40" s="12" t="n">
+      <c r="E40" s="13" t="n">
         <v>450000</v>
       </c>
-      <c r="F40" s="12" t="n">
+      <c r="F40" s="13" t="n">
         <v>850000</v>
       </c>
-      <c r="G40" s="12" t="n">
+      <c r="G40" s="13" t="n">
         <v>1400000</v>
       </c>
     </row>
@@ -3054,24 +3054,24 @@
           <t>Enterprise Tools, Security Audits &amp; G&amp;A Infrastructure</t>
         </is>
       </c>
-      <c r="C41" s="12" t="n">
+      <c r="C41" s="13" t="n">
         <v>70000</v>
       </c>
-      <c r="D41" s="12" t="n">
+      <c r="D41" s="13" t="n">
         <v>150000</v>
       </c>
-      <c r="E41" s="12" t="n">
+      <c r="E41" s="13" t="n">
         <v>320000</v>
       </c>
-      <c r="F41" s="12" t="n">
+      <c r="F41" s="13" t="n">
         <v>580000</v>
       </c>
-      <c r="G41" s="12" t="n">
+      <c r="G41" s="13" t="n">
         <v>920000</v>
       </c>
     </row>
     <row r="42">
-      <c r="B42" s="13" t="inlineStr">
+      <c r="B42" s="14" t="inlineStr">
         <is>
           <t>TOTAL OPERATING EXPENSES</t>
         </is>
@@ -3106,7 +3106,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="B45" s="13" t="inlineStr">
+      <c r="B45" s="14" t="inlineStr">
         <is>
           <t>EBITDA (OPERATING PROFIT)</t>
         </is>
@@ -3133,7 +3133,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="B46" s="13" t="inlineStr">
+      <c r="B46" s="14" t="inlineStr">
         <is>
           <t>EBITDA Margin %</t>
         </is>
@@ -3165,19 +3165,19 @@
           <t>Less: Depreciation &amp; Amortization (Servers/Hardware)</t>
         </is>
       </c>
-      <c r="C47" s="12" t="n">
+      <c r="C47" s="13" t="n">
         <v>24000</v>
       </c>
-      <c r="D47" s="12" t="n">
+      <c r="D47" s="13" t="n">
         <v>52000</v>
       </c>
-      <c r="E47" s="12" t="n">
+      <c r="E47" s="13" t="n">
         <v>110000</v>
       </c>
-      <c r="F47" s="12" t="n">
+      <c r="F47" s="13" t="n">
         <v>210000</v>
       </c>
-      <c r="G47" s="12" t="n">
+      <c r="G47" s="13" t="n">
         <v>350000</v>
       </c>
     </row>
@@ -3187,23 +3187,23 @@
           <t>Operating Income (EBIT)</t>
         </is>
       </c>
-      <c r="C48" s="12">
+      <c r="C48" s="13">
         <f>C45-C47</f>
         <v/>
       </c>
-      <c r="D48" s="12">
+      <c r="D48" s="13">
         <f>D45-D47</f>
         <v/>
       </c>
-      <c r="E48" s="12">
+      <c r="E48" s="13">
         <f>E45-E47</f>
         <v/>
       </c>
-      <c r="F48" s="12">
+      <c r="F48" s="13">
         <f>F45-F47</f>
         <v/>
       </c>
-      <c r="G48" s="12">
+      <c r="G48" s="13">
         <f>G45-G47</f>
         <v/>
       </c>
@@ -3214,19 +3214,19 @@
           <t>Net Interest Income (Treasury Cash Reserve Yield @ 4.8%)</t>
         </is>
       </c>
-      <c r="C49" s="16" t="n">
+      <c r="C49" s="13" t="n">
         <v>134400</v>
       </c>
-      <c r="D49" s="16" t="n">
+      <c r="D49" s="13" t="n">
         <v>115000</v>
       </c>
-      <c r="E49" s="16" t="n">
+      <c r="E49" s="13" t="n">
         <v>280000</v>
       </c>
-      <c r="F49" s="16" t="n">
+      <c r="F49" s="13" t="n">
         <v>650000</v>
       </c>
-      <c r="G49" s="16" t="n">
+      <c r="G49" s="13" t="n">
         <v>1420000</v>
       </c>
     </row>
@@ -3236,23 +3236,23 @@
           <t>Earnings Before Taxes (EBT)</t>
         </is>
       </c>
-      <c r="C50" s="12">
+      <c r="C50" s="13">
         <f>C48+C49</f>
         <v/>
       </c>
-      <c r="D50" s="12">
+      <c r="D50" s="13">
         <f>D48+D49</f>
         <v/>
       </c>
-      <c r="E50" s="12">
+      <c r="E50" s="13">
         <f>E48+E49</f>
         <v/>
       </c>
-      <c r="F50" s="12">
+      <c r="F50" s="13">
         <f>F48+F49</f>
         <v/>
       </c>
-      <c r="G50" s="12">
+      <c r="G50" s="13">
         <f>G48+G49</f>
         <v/>
       </c>
@@ -3263,29 +3263,29 @@
           <t>Income Tax Expense (21% Federal/State Effective)</t>
         </is>
       </c>
-      <c r="C51" s="16">
+      <c r="C51" s="13">
         <f>IF(C50&gt;0, C50*0.21, 0)</f>
         <v/>
       </c>
-      <c r="D51" s="16">
+      <c r="D51" s="13">
         <f>IF(D50&gt;0, D50*0.21, 0)</f>
         <v/>
       </c>
-      <c r="E51" s="16">
+      <c r="E51" s="13">
         <f>IF(E50&gt;0, E50*0.21, 0)</f>
         <v/>
       </c>
-      <c r="F51" s="16">
+      <c r="F51" s="13">
         <f>IF(F50&gt;0, F50*0.21, 0)</f>
         <v/>
       </c>
-      <c r="G51" s="16">
+      <c r="G51" s="13">
         <f>IF(G50&gt;0, G50*0.21, 0)</f>
         <v/>
       </c>
     </row>
     <row r="52">
-      <c r="B52" s="13" t="inlineStr">
+      <c r="B52" s="14" t="inlineStr">
         <is>
           <t>NET INCOME (AFTER-TAX PROFIT)</t>
         </is>
@@ -3317,23 +3317,23 @@
           <t>Net Income Margin %</t>
         </is>
       </c>
-      <c r="C53" s="16">
+      <c r="C53" s="17">
         <f>C52/C26</f>
         <v/>
       </c>
-      <c r="D53" s="16">
+      <c r="D53" s="17">
         <f>D52/D26</f>
         <v/>
       </c>
-      <c r="E53" s="16">
+      <c r="E53" s="17">
         <f>E52/E26</f>
         <v/>
       </c>
-      <c r="F53" s="16">
+      <c r="F53" s="17">
         <f>F52/F26</f>
         <v/>
       </c>
-      <c r="G53" s="16">
+      <c r="G53" s="17">
         <f>G52/G26</f>
         <v/>
       </c>
@@ -3459,55 +3459,55 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>Beginning Cash Balance</t>
         </is>
       </c>
-      <c r="C6" s="14" t="n">
+      <c r="C6" s="15" t="n">
         <v>3500000</v>
       </c>
-      <c r="D6" s="14">
+      <c r="D6" s="15">
         <f>C26</f>
         <v/>
       </c>
-      <c r="E6" s="14">
+      <c r="E6" s="15">
         <f>D26</f>
         <v/>
       </c>
-      <c r="F6" s="14">
+      <c r="F6" s="15">
         <f>E26</f>
         <v/>
       </c>
-      <c r="G6" s="14">
+      <c r="G6" s="15">
         <f>F26</f>
         <v/>
       </c>
-      <c r="H6" s="14">
+      <c r="H6" s="15">
         <f>G26</f>
         <v/>
       </c>
-      <c r="I6" s="14">
+      <c r="I6" s="15">
         <f>H26</f>
         <v/>
       </c>
-      <c r="J6" s="14">
+      <c r="J6" s="15">
         <f>I26</f>
         <v/>
       </c>
-      <c r="K6" s="14">
+      <c r="K6" s="15">
         <f>J26</f>
         <v/>
       </c>
-      <c r="L6" s="14">
+      <c r="L6" s="15">
         <f>K26</f>
         <v/>
       </c>
-      <c r="M6" s="14">
+      <c r="M6" s="15">
         <f>L26</f>
         <v/>
       </c>
-      <c r="N6" s="14">
+      <c r="N6" s="15">
         <f>M26</f>
         <v/>
       </c>
@@ -3521,7 +3521,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>Active Client Desks</t>
         </is>
@@ -3564,203 +3564,203 @@
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>Monthly Subscription Inflows</t>
         </is>
       </c>
-      <c r="C10" s="12">
-        <f>C9*'Model Assumptions'!C16</f>
-        <v/>
-      </c>
-      <c r="D10" s="12">
-        <f>D9*'Model Assumptions'!C16</f>
-        <v/>
-      </c>
-      <c r="E10" s="12">
-        <f>E9*'Model Assumptions'!C16</f>
-        <v/>
-      </c>
-      <c r="F10" s="12">
-        <f>F9*'Model Assumptions'!C16</f>
-        <v/>
-      </c>
-      <c r="G10" s="12">
-        <f>G9*'Model Assumptions'!C16</f>
-        <v/>
-      </c>
-      <c r="H10" s="12">
-        <f>H9*'Model Assumptions'!C16</f>
-        <v/>
-      </c>
-      <c r="I10" s="12">
-        <f>I9*'Model Assumptions'!C16</f>
-        <v/>
-      </c>
-      <c r="J10" s="12">
-        <f>J9*'Model Assumptions'!C16</f>
-        <v/>
-      </c>
-      <c r="K10" s="12">
-        <f>K9*'Model Assumptions'!C16</f>
-        <v/>
-      </c>
-      <c r="L10" s="12">
-        <f>L9*'Model Assumptions'!C16</f>
-        <v/>
-      </c>
-      <c r="M10" s="12">
-        <f>M9*'Model Assumptions'!C16</f>
-        <v/>
-      </c>
-      <c r="N10" s="12">
-        <f>N9*'Model Assumptions'!C16</f>
+      <c r="C10" s="13">
+        <f>C9*'Model Assumptions'!C17</f>
+        <v/>
+      </c>
+      <c r="D10" s="13">
+        <f>D9*'Model Assumptions'!C17</f>
+        <v/>
+      </c>
+      <c r="E10" s="13">
+        <f>E9*'Model Assumptions'!C17</f>
+        <v/>
+      </c>
+      <c r="F10" s="13">
+        <f>F9*'Model Assumptions'!C17</f>
+        <v/>
+      </c>
+      <c r="G10" s="13">
+        <f>G9*'Model Assumptions'!C17</f>
+        <v/>
+      </c>
+      <c r="H10" s="13">
+        <f>H9*'Model Assumptions'!C17</f>
+        <v/>
+      </c>
+      <c r="I10" s="13">
+        <f>I9*'Model Assumptions'!C17</f>
+        <v/>
+      </c>
+      <c r="J10" s="13">
+        <f>J9*'Model Assumptions'!C17</f>
+        <v/>
+      </c>
+      <c r="K10" s="13">
+        <f>K9*'Model Assumptions'!C17</f>
+        <v/>
+      </c>
+      <c r="L10" s="13">
+        <f>L9*'Model Assumptions'!C17</f>
+        <v/>
+      </c>
+      <c r="M10" s="13">
+        <f>M9*'Model Assumptions'!C17</f>
+        <v/>
+      </c>
+      <c r="N10" s="13">
+        <f>N9*'Model Assumptions'!C17</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="14" t="inlineStr">
         <is>
           <t>Annual Upfront Prepay Cash Float</t>
         </is>
       </c>
-      <c r="C11" s="12" t="n">
+      <c r="C11" s="13" t="n">
         <v>122400</v>
       </c>
-      <c r="D11" s="12" t="n">
+      <c r="D11" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="12" t="n">
+      <c r="E11" s="13" t="n">
         <v>122400</v>
       </c>
-      <c r="F11" s="12" t="n">
+      <c r="F11" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="12" t="n">
+      <c r="G11" s="13" t="n">
         <v>122400</v>
       </c>
-      <c r="H11" s="12" t="n">
+      <c r="H11" s="13" t="n">
         <v>122400</v>
       </c>
-      <c r="I11" s="12" t="n">
+      <c r="I11" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="J11" s="12" t="n">
+      <c r="J11" s="13" t="n">
         <v>122400</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="K11" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="L11" s="12" t="n">
+      <c r="L11" s="13" t="n">
         <v>122400</v>
       </c>
-      <c r="M11" s="12" t="n">
+      <c r="M11" s="13" t="n">
         <v>122400</v>
       </c>
-      <c r="N11" s="12" t="n">
+      <c r="N11" s="13" t="n">
         <v>122400</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="14" t="inlineStr">
         <is>
           <t>Variable Volume Routing Fees</t>
         </is>
       </c>
-      <c r="C12" s="12" t="n">
+      <c r="C12" s="13" t="n">
         <v>2500</v>
       </c>
-      <c r="D12" s="12" t="n">
+      <c r="D12" s="13" t="n">
         <v>3200</v>
       </c>
-      <c r="E12" s="12" t="n">
+      <c r="E12" s="13" t="n">
         <v>5400</v>
       </c>
-      <c r="F12" s="12" t="n">
+      <c r="F12" s="13" t="n">
         <v>7800</v>
       </c>
-      <c r="G12" s="12" t="n">
+      <c r="G12" s="13" t="n">
         <v>10500</v>
       </c>
-      <c r="H12" s="12" t="n">
+      <c r="H12" s="13" t="n">
         <v>13200</v>
       </c>
-      <c r="I12" s="12" t="n">
+      <c r="I12" s="13" t="n">
         <v>16800</v>
       </c>
-      <c r="J12" s="12" t="n">
+      <c r="J12" s="13" t="n">
         <v>20400</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="K12" s="13" t="n">
         <v>24500</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="L12" s="13" t="n">
         <v>29000</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="M12" s="13" t="n">
         <v>34000</v>
       </c>
-      <c r="N12" s="12" t="n">
+      <c r="N12" s="13" t="n">
         <v>41000</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B13" s="14" t="inlineStr">
         <is>
           <t>Treasury Yield (Cash Sweep @ 4.8%)</t>
         </is>
       </c>
-      <c r="C13" s="12">
+      <c r="C13" s="13">
         <f>C6*0.048/12</f>
         <v/>
       </c>
-      <c r="D13" s="12">
+      <c r="D13" s="13">
         <f>D6*0.048/12</f>
         <v/>
       </c>
-      <c r="E13" s="12">
+      <c r="E13" s="13">
         <f>E6*0.048/12</f>
         <v/>
       </c>
-      <c r="F13" s="12">
+      <c r="F13" s="13">
         <f>F6*0.048/12</f>
         <v/>
       </c>
-      <c r="G13" s="12">
+      <c r="G13" s="13">
         <f>G6*0.048/12</f>
         <v/>
       </c>
-      <c r="H13" s="12">
+      <c r="H13" s="13">
         <f>H6*0.048/12</f>
         <v/>
       </c>
-      <c r="I13" s="12">
+      <c r="I13" s="13">
         <f>I6*0.048/12</f>
         <v/>
       </c>
-      <c r="J13" s="12">
+      <c r="J13" s="13">
         <f>J6*0.048/12</f>
         <v/>
       </c>
-      <c r="K13" s="12">
+      <c r="K13" s="13">
         <f>K6*0.048/12</f>
         <v/>
       </c>
-      <c r="L13" s="12">
+      <c r="L13" s="13">
         <f>L6*0.048/12</f>
         <v/>
       </c>
-      <c r="M13" s="12">
+      <c r="M13" s="13">
         <f>M6*0.048/12</f>
         <v/>
       </c>
-      <c r="N13" s="12">
+      <c r="N13" s="13">
         <f>N6*0.048/12</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B14" s="14" t="inlineStr">
         <is>
           <t>Total Monthly Cash Inflows</t>
         </is>
@@ -3823,222 +3823,222 @@
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B17" s="14" t="inlineStr">
         <is>
           <t>Infrastructure &amp; Co-Location COGS</t>
         </is>
       </c>
-      <c r="C17" s="12" t="n">
+      <c r="C17" s="13" t="n">
         <v>11200</v>
       </c>
-      <c r="D17" s="12" t="n">
+      <c r="D17" s="13" t="n">
         <v>11200</v>
       </c>
-      <c r="E17" s="12" t="n">
+      <c r="E17" s="13" t="n">
         <v>12400</v>
       </c>
-      <c r="F17" s="12" t="n">
+      <c r="F17" s="13" t="n">
         <v>12400</v>
       </c>
-      <c r="G17" s="12" t="n">
+      <c r="G17" s="13" t="n">
         <v>13600</v>
       </c>
-      <c r="H17" s="12" t="n">
+      <c r="H17" s="13" t="n">
         <v>13600</v>
       </c>
-      <c r="I17" s="12" t="n">
+      <c r="I17" s="13" t="n">
         <v>14800</v>
       </c>
-      <c r="J17" s="12" t="n">
+      <c r="J17" s="13" t="n">
         <v>14800</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="K17" s="13" t="n">
         <v>16000</v>
       </c>
-      <c r="L17" s="12" t="n">
+      <c r="L17" s="13" t="n">
         <v>16000</v>
       </c>
-      <c r="M17" s="12" t="n">
+      <c r="M17" s="13" t="n">
         <v>17200</v>
       </c>
-      <c r="N17" s="12" t="n">
+      <c r="N17" s="13" t="n">
         <v>17200</v>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B18" s="14" t="inlineStr">
         <is>
           <t>Engineering Payroll (4 Engineers)</t>
         </is>
       </c>
-      <c r="C18" s="12" t="n">
+      <c r="C18" s="13" t="n">
         <v>70000</v>
       </c>
-      <c r="D18" s="12" t="n">
+      <c r="D18" s="13" t="n">
         <v>70000</v>
       </c>
-      <c r="E18" s="12" t="n">
+      <c r="E18" s="13" t="n">
         <v>70000</v>
       </c>
-      <c r="F18" s="12" t="n">
+      <c r="F18" s="13" t="n">
         <v>70000</v>
       </c>
-      <c r="G18" s="12" t="n">
+      <c r="G18" s="13" t="n">
         <v>70000</v>
       </c>
-      <c r="H18" s="12" t="n">
+      <c r="H18" s="13" t="n">
         <v>70000</v>
       </c>
-      <c r="I18" s="12" t="n">
+      <c r="I18" s="13" t="n">
         <v>70000</v>
       </c>
-      <c r="J18" s="12" t="n">
+      <c r="J18" s="13" t="n">
         <v>70000</v>
       </c>
-      <c r="K18" s="12" t="n">
+      <c r="K18" s="13" t="n">
         <v>70000</v>
       </c>
-      <c r="L18" s="12" t="n">
+      <c r="L18" s="13" t="n">
         <v>70000</v>
       </c>
-      <c r="M18" s="12" t="n">
+      <c r="M18" s="13" t="n">
         <v>70000</v>
       </c>
-      <c r="N18" s="12" t="n">
+      <c r="N18" s="13" t="n">
         <v>70000</v>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="13" t="inlineStr">
+      <c r="B19" s="14" t="inlineStr">
         <is>
           <t>Sales &amp; Business Development</t>
         </is>
       </c>
-      <c r="C19" s="12" t="n">
+      <c r="C19" s="13" t="n">
         <v>12000</v>
       </c>
-      <c r="D19" s="12" t="n">
+      <c r="D19" s="13" t="n">
         <v>12000</v>
       </c>
-      <c r="E19" s="12" t="n">
+      <c r="E19" s="13" t="n">
         <v>15000</v>
       </c>
-      <c r="F19" s="12" t="n">
+      <c r="F19" s="13" t="n">
         <v>15000</v>
       </c>
-      <c r="G19" s="12" t="n">
+      <c r="G19" s="13" t="n">
         <v>18000</v>
       </c>
-      <c r="H19" s="12" t="n">
+      <c r="H19" s="13" t="n">
         <v>18000</v>
       </c>
-      <c r="I19" s="12" t="n">
+      <c r="I19" s="13" t="n">
         <v>21000</v>
       </c>
-      <c r="J19" s="12" t="n">
+      <c r="J19" s="13" t="n">
         <v>21000</v>
       </c>
-      <c r="K19" s="12" t="n">
+      <c r="K19" s="13" t="n">
         <v>24000</v>
       </c>
-      <c r="L19" s="12" t="n">
+      <c r="L19" s="13" t="n">
         <v>24000</v>
       </c>
-      <c r="M19" s="12" t="n">
+      <c r="M19" s="13" t="n">
         <v>27000</v>
       </c>
-      <c r="N19" s="12" t="n">
+      <c r="N19" s="13" t="n">
         <v>27000</v>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="13" t="inlineStr">
+      <c r="B20" s="14" t="inlineStr">
         <is>
           <t>Legal, Compliance &amp; Retainers</t>
         </is>
       </c>
-      <c r="C20" s="12" t="n">
+      <c r="C20" s="13" t="n">
         <v>15000</v>
       </c>
-      <c r="D20" s="12" t="n">
+      <c r="D20" s="13" t="n">
         <v>6000</v>
       </c>
-      <c r="E20" s="12" t="n">
+      <c r="E20" s="13" t="n">
         <v>6000</v>
       </c>
-      <c r="F20" s="12" t="n">
+      <c r="F20" s="13" t="n">
         <v>6000</v>
       </c>
-      <c r="G20" s="12" t="n">
+      <c r="G20" s="13" t="n">
         <v>6000</v>
       </c>
-      <c r="H20" s="12" t="n">
+      <c r="H20" s="13" t="n">
         <v>6000</v>
       </c>
-      <c r="I20" s="12" t="n">
+      <c r="I20" s="13" t="n">
         <v>6000</v>
       </c>
-      <c r="J20" s="12" t="n">
+      <c r="J20" s="13" t="n">
         <v>6000</v>
       </c>
-      <c r="K20" s="12" t="n">
+      <c r="K20" s="13" t="n">
         <v>6000</v>
       </c>
-      <c r="L20" s="12" t="n">
+      <c r="L20" s="13" t="n">
         <v>6000</v>
       </c>
-      <c r="M20" s="12" t="n">
+      <c r="M20" s="13" t="n">
         <v>6000</v>
       </c>
-      <c r="N20" s="12" t="n">
+      <c r="N20" s="13" t="n">
         <v>6000</v>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B21" s="14" t="inlineStr">
         <is>
           <t>SaaS Tooling, Admin, Insurance</t>
         </is>
       </c>
-      <c r="C21" s="12" t="n">
+      <c r="C21" s="13" t="n">
         <v>4500</v>
       </c>
-      <c r="D21" s="12" t="n">
+      <c r="D21" s="13" t="n">
         <v>4500</v>
       </c>
-      <c r="E21" s="12" t="n">
+      <c r="E21" s="13" t="n">
         <v>4800</v>
       </c>
-      <c r="F21" s="12" t="n">
+      <c r="F21" s="13" t="n">
         <v>4800</v>
       </c>
-      <c r="G21" s="12" t="n">
+      <c r="G21" s="13" t="n">
         <v>5200</v>
       </c>
-      <c r="H21" s="12" t="n">
+      <c r="H21" s="13" t="n">
         <v>5200</v>
       </c>
-      <c r="I21" s="12" t="n">
+      <c r="I21" s="13" t="n">
         <v>5600</v>
       </c>
-      <c r="J21" s="12" t="n">
+      <c r="J21" s="13" t="n">
         <v>5600</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="K21" s="13" t="n">
         <v>6000</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="L21" s="13" t="n">
         <v>6000</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="M21" s="13" t="n">
         <v>6500</v>
       </c>
-      <c r="N21" s="12" t="n">
+      <c r="N21" s="13" t="n">
         <v>6500</v>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B22" s="14" t="inlineStr">
         <is>
           <t>Total Monthly Cash Outflows</t>
         </is>
@@ -4094,7 +4094,7 @@
     </row>
     <row r="23"/>
     <row r="24">
-      <c r="B24" s="13" t="inlineStr">
+      <c r="B24" s="14" t="inlineStr">
         <is>
           <t>NET MONTHLY CASH FLOW</t>
         </is>
@@ -4150,7 +4150,7 @@
     </row>
     <row r="25"/>
     <row r="26">
-      <c r="B26" s="13" t="inlineStr">
+      <c r="B26" s="14" t="inlineStr">
         <is>
           <t>ENDING CASH BALANCE</t>
         </is>
@@ -4205,7 +4205,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="13" t="inlineStr">
+      <c r="B27" s="14" t="inlineStr">
         <is>
           <t>Runway Remaining (Months at Gross Burn)</t>
         </is>
@@ -4338,16 +4338,16 @@
           <t>Annual Contract Value (ACV)</t>
         </is>
       </c>
-      <c r="C7" s="12" t="n">
+      <c r="C7" s="13" t="n">
         <v>30000</v>
       </c>
-      <c r="D7" s="12" t="n">
+      <c r="D7" s="13" t="n">
         <v>144000</v>
       </c>
-      <c r="E7" s="12" t="n">
+      <c r="E7" s="13" t="n">
         <v>420000</v>
       </c>
-      <c r="F7" s="12" t="n">
+      <c r="F7" s="13" t="n">
         <v>162000</v>
       </c>
     </row>
@@ -4357,21 +4357,21 @@
           <t>Customer Acquisition Cost (CAC)</t>
         </is>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="C8" s="13" t="n">
         <v>12000</v>
       </c>
-      <c r="D8" s="12" t="n">
+      <c r="D8" s="13" t="n">
         <v>22000</v>
       </c>
-      <c r="E8" s="12" t="n">
+      <c r="E8" s="13" t="n">
         <v>65000</v>
       </c>
-      <c r="F8" s="12" t="n">
+      <c r="F8" s="13" t="n">
         <v>28000</v>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>Payback Period (Months)</t>
         </is>
@@ -4399,16 +4399,16 @@
           <t>Gross Margin Contribution %</t>
         </is>
       </c>
-      <c r="C10" s="16" t="n">
+      <c r="C10" s="17" t="n">
         <v>0.92</v>
       </c>
-      <c r="D10" s="16" t="n">
+      <c r="D10" s="17" t="n">
         <v>0.9399999999999999</v>
       </c>
-      <c r="E10" s="16" t="n">
+      <c r="E10" s="17" t="n">
         <v>0.96</v>
       </c>
-      <c r="F10" s="16" t="n">
+      <c r="F10" s="17" t="n">
         <v>0.9399999999999999</v>
       </c>
     </row>
@@ -4418,16 +4418,16 @@
           <t>Annual Churn Rate %</t>
         </is>
       </c>
-      <c r="C11" s="16" t="n">
+      <c r="C11" s="17" t="n">
         <v>0.08</v>
       </c>
-      <c r="D11" s="16" t="n">
+      <c r="D11" s="17" t="n">
         <v>0.04</v>
       </c>
-      <c r="E11" s="16" t="n">
+      <c r="E11" s="17" t="n">
         <v>0.02</v>
       </c>
-      <c r="F11" s="16" t="n">
+      <c r="F11" s="17" t="n">
         <v>0.045</v>
       </c>
     </row>
@@ -4460,25 +4460,25 @@
           <t>Lifetime Value (LTV)</t>
         </is>
       </c>
-      <c r="C13" s="12">
+      <c r="C13" s="13">
         <f>C7*C10*C12</f>
         <v/>
       </c>
-      <c r="D13" s="12">
+      <c r="D13" s="13">
         <f>D7*D10*D12</f>
         <v/>
       </c>
-      <c r="E13" s="12">
+      <c r="E13" s="13">
         <f>E7*E10*E12</f>
         <v/>
       </c>
-      <c r="F13" s="12">
+      <c r="F13" s="13">
         <f>F7*F10*F12</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B14" s="14" t="inlineStr">
         <is>
           <t>LTV / CAC Ratio</t>
         </is>
@@ -4542,61 +4542,61 @@
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="13" t="inlineStr">
+      <c r="B19" s="14" t="inlineStr">
         <is>
           <t>15x Forward ARR Multiple</t>
         </is>
       </c>
-      <c r="C19" s="12">
+      <c r="C19" s="13">
         <f>'5-Year Pro-Forma'!C26*15.0</f>
         <v/>
       </c>
-      <c r="D19" s="12">
+      <c r="D19" s="13">
         <f>'5-Year Pro-Forma'!D26*15.0</f>
         <v/>
       </c>
-      <c r="E19" s="12">
+      <c r="E19" s="13">
         <f>'5-Year Pro-Forma'!E26*15.0</f>
         <v/>
       </c>
-      <c r="F19" s="12">
+      <c r="F19" s="13">
         <f>'5-Year Pro-Forma'!F26*15.0</f>
         <v/>
       </c>
-      <c r="G19" s="12">
+      <c r="G19" s="13">
         <f>'5-Year Pro-Forma'!G26*15.0</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="13" t="inlineStr">
+      <c r="B20" s="14" t="inlineStr">
         <is>
           <t>20x Forward ARR Multiple</t>
         </is>
       </c>
-      <c r="C20" s="12">
+      <c r="C20" s="13">
         <f>'5-Year Pro-Forma'!C26*20.0</f>
         <v/>
       </c>
-      <c r="D20" s="12">
+      <c r="D20" s="13">
         <f>'5-Year Pro-Forma'!D26*20.0</f>
         <v/>
       </c>
-      <c r="E20" s="12">
+      <c r="E20" s="13">
         <f>'5-Year Pro-Forma'!E26*20.0</f>
         <v/>
       </c>
-      <c r="F20" s="12">
+      <c r="F20" s="13">
         <f>'5-Year Pro-Forma'!F26*20.0</f>
         <v/>
       </c>
-      <c r="G20" s="12">
+      <c r="G20" s="13">
         <f>'5-Year Pro-Forma'!G26*20.0</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B21" s="14" t="inlineStr">
         <is>
           <t>25x Forward ARR Multiple</t>
         </is>
@@ -4623,55 +4623,55 @@
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B22" s="14" t="inlineStr">
         <is>
           <t>30x Forward ARR Multiple</t>
         </is>
       </c>
-      <c r="C22" s="12">
+      <c r="C22" s="13">
         <f>'5-Year Pro-Forma'!C26*30.0</f>
         <v/>
       </c>
-      <c r="D22" s="12">
+      <c r="D22" s="13">
         <f>'5-Year Pro-Forma'!D26*30.0</f>
         <v/>
       </c>
-      <c r="E22" s="12">
+      <c r="E22" s="13">
         <f>'5-Year Pro-Forma'!E26*30.0</f>
         <v/>
       </c>
-      <c r="F22" s="12">
+      <c r="F22" s="13">
         <f>'5-Year Pro-Forma'!F26*30.0</f>
         <v/>
       </c>
-      <c r="G22" s="12">
+      <c r="G22" s="13">
         <f>'5-Year Pro-Forma'!G26*30.0</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="13" t="inlineStr">
+      <c r="B23" s="14" t="inlineStr">
         <is>
           <t>35x Forward ARR Multiple</t>
         </is>
       </c>
-      <c r="C23" s="12">
+      <c r="C23" s="13">
         <f>'5-Year Pro-Forma'!C26*35.0</f>
         <v/>
       </c>
-      <c r="D23" s="12">
+      <c r="D23" s="13">
         <f>'5-Year Pro-Forma'!D26*35.0</f>
         <v/>
       </c>
-      <c r="E23" s="12">
+      <c r="E23" s="13">
         <f>'5-Year Pro-Forma'!E26*35.0</f>
         <v/>
       </c>
-      <c r="F23" s="12">
+      <c r="F23" s="13">
         <f>'5-Year Pro-Forma'!F26*35.0</f>
         <v/>
       </c>
-      <c r="G23" s="12">
+      <c r="G23" s="13">
         <f>'5-Year Pro-Forma'!G26*35.0</f>
         <v/>
       </c>
@@ -4708,7 +4708,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="13" t="inlineStr">
+      <c r="B28" s="14" t="inlineStr">
         <is>
           <t>Intercontinental Exchange (ICE / NYSE)</t>
         </is>
@@ -4718,7 +4718,7 @@
           <t>Acquisition of primary cross-venue event derivative routing utility</t>
         </is>
       </c>
-      <c r="D28" s="21" t="inlineStr">
+      <c r="D28" s="22" t="inlineStr">
         <is>
           <t>ICE acquired Ellie Mae ($11B) &amp; SuperDerivatives ($350M)</t>
         </is>
@@ -4730,7 +4730,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="13" t="inlineStr">
+      <c r="B29" s="14" t="inlineStr">
         <is>
           <t>Bloomberg LP / Tradebook</t>
         </is>
@@ -4740,7 +4740,7 @@
           <t>Incorporation into 350k+ Bloomberg Terminals as native event execution engine</t>
         </is>
       </c>
-      <c r="D29" s="21" t="inlineStr">
+      <c r="D29" s="22" t="inlineStr">
         <is>
           <t>Bloomberg acquisitions of EMS/OEMS utilities</t>
         </is>
@@ -4752,7 +4752,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="13" t="inlineStr">
+      <c r="B30" s="14" t="inlineStr">
         <is>
           <t>CME Group</t>
         </is>
@@ -4762,7 +4762,7 @@
           <t>Integration with CME Event Contracts to dominate institutional macro derivative flow</t>
         </is>
       </c>
-      <c r="D30" s="21" t="inlineStr">
+      <c r="D30" s="22" t="inlineStr">
         <is>
           <t>CME acquired NEX Group ($5.5B)</t>
         </is>
@@ -4774,7 +4774,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="13" t="inlineStr">
+      <c r="B31" s="14" t="inlineStr">
         <is>
           <t>Citadel Securities / Jane Street</t>
         </is>
@@ -4784,7 +4784,7 @@
           <t>Internalization of high-value non-toxic institutional event flow</t>
         </is>
       </c>
-      <c r="D31" s="21" t="inlineStr">
+      <c r="D31" s="22" t="inlineStr">
         <is>
           <t>Virtu acquired ITG ($1B)</t>
         </is>
@@ -4796,7 +4796,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="13" t="inlineStr">
+      <c r="B32" s="14" t="inlineStr">
         <is>
           <t>Coinbase Institutional</t>
         </is>
@@ -4806,7 +4806,7 @@
           <t>Expansion from crypto spot/perps into global regulated event prediction markets</t>
         </is>
       </c>
-      <c r="D32" s="21" t="inlineStr">
+      <c r="D32" s="22" t="inlineStr">
         <is>
           <t>Coinbase acquired Tagomi ($100M+)</t>
         </is>

</xml_diff>